<commit_message>
update data from excel
</commit_message>
<xml_diff>
--- a/scripts/gripic_data.xlsx
+++ b/scripts/gripic_data.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="68">
   <si>
     <t xml:space="preserve">nom</t>
   </si>
@@ -151,6 +151,39 @@
     <t xml:space="preserve">content related to Autres</t>
   </si>
   <si>
+    <t xml:space="preserve">Projets en cours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projets de recherche</t>
+  </si>
+  <si>
+    <t xml:space="preserve">content related to Projets en cours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projets passés</t>
+  </si>
+  <si>
+    <t xml:space="preserve">content related to Projets de recherche</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partenariats et participations internes à Sorbonne université</t>
+  </si>
+  <si>
+    <t xml:space="preserve">content related to Partenariats internes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partenariats externes (institutions, entreprises, fondations)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">content related to Partenariats externes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programmes passés</t>
+  </si>
+  <si>
+    <t xml:space="preserve">content related to Programmes passés : parapluie</t>
+  </si>
+  <si>
     <t xml:space="preserve">Master "Communication en transformation"</t>
   </si>
   <si>
@@ -187,10 +220,10 @@
     <t xml:space="preserve">gabo papasito</t>
   </si>
   <si>
-    <t xml:space="preserve">Test 2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bla bla bla</t>
+    <t xml:space="preserve">vgvkjbkh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a ver </t>
   </si>
 </sst>
 </file>
@@ -789,34 +822,99 @@
         <v>52</v>
       </c>
       <c r="B23" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23" s="1" t="s">
         <v>53</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B24" s="1" t="s">
-        <v>53</v>
-      </c>
       <c r="C24" s="1" t="s">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="1048567" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048568" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048569" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048570" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
-    <row r="1048571" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
     <row r="1048572" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048573" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
     <row r="1048574" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>

</xml_diff>